<commit_message>
Automatic update of files.
</commit_message>
<xml_diff>
--- a/Översikt UPPLANDS VÄSBY.xlsx
+++ b/Översikt UPPLANDS VÄSBY.xlsx
@@ -601,7 +601,7 @@
         <v>46056</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
         <v>45806</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -813,7 +813,7 @@
         <v>44571</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -869,7 +869,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
-          <t>A 27724-2022</t>
+          <t>A 50934-2024</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -883,10 +883,10 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>44743</v>
+        <v>45602</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -942,7 +942,7 @@
     <row r="6" ht="15" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A 31120-2023</t>
+          <t>A 16862-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -952,14 +952,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Avverkning för annat ändamål</t>
+          <t>Föryngringsavverkning</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>45113</v>
+        <v>46113</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>0.2</v>
+        <v>3.9</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -1032,7 +1032,7 @@
         <v>46113</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1088,7 +1088,7 @@
     <row r="8" ht="15" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A 16862-2026</t>
+          <t>A 56917-2025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1102,10 +1102,10 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46113</v>
+        <v>45978</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1118,7 +1118,7 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>3.9</v>
+        <v>0.7</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -1161,7 +1161,7 @@
     <row r="9" ht="15" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A 56917-2025</t>
+          <t>A 31120-2023</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1171,14 +1171,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Föryngringsavverkning</t>
+          <t>Avverkning för annat ändamål</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>45978</v>
+        <v>45113</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -1234,7 +1234,7 @@
     <row r="10" ht="15" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
-          <t>A 64431-2023</t>
+          <t>A 20900-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1248,10 +1248,10 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>45280</v>
+        <v>46142</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1264,7 +1264,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -1307,7 +1307,7 @@
     <row r="11" ht="15" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A 20900-2026</t>
+          <t>A 64431-2023</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1321,10 +1321,10 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46142</v>
+        <v>45280</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -1380,7 +1380,7 @@
     <row r="12" ht="15" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
-          <t>A 8748-2022</t>
+          <t>A 27724-2022</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1394,10 +1394,10 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>44613</v>
+        <v>44743</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -1453,7 +1453,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>A 50934-2024</t>
+          <t>A 8748-2022</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1467,10 +1467,10 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>45602</v>
+        <v>44613</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>

</xml_diff>